<commit_message>
fixed a few bugs
</commit_message>
<xml_diff>
--- a/Assets/Spreadsheets/GunBalancing.xlsx
+++ b/Assets/Spreadsheets/GunBalancing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zilant\Unity Projects SSD\Jam Game\Assets\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A88530-B51B-47F1-972A-57CB58C6293F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D6A73A9-453B-4A2D-A313-B3EEBA8C5702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="375" yWindow="2055" windowWidth="28800" windowHeight="18450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -116,9 +116,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -162,19 +161,19 @@
     <tableColumn id="4" xr3:uid="{54FA7190-3A01-4900-8896-7ECBE5F2B001}" name="Bullets/Shot"/>
     <tableColumn id="6" xr3:uid="{21CBDCD8-D87A-425D-A824-26263FE395B9}" name="Mag size"/>
     <tableColumn id="8" xr3:uid="{D4CDCDB1-AB63-46BA-A487-5E8206D2F9E1}" name="Mag count"/>
-    <tableColumn id="11" xr3:uid="{6B6D3C5F-49E9-4742-BF69-34AE1A9C53B3}" name="Spare ammo count" dataDxfId="1">
+    <tableColumn id="11" xr3:uid="{6B6D3C5F-49E9-4742-BF69-34AE1A9C53B3}" name="Spare ammo count" dataDxfId="4">
       <calculatedColumnFormula>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{3136763A-E7B4-4737-8D7B-5551B327F9C1}" name="Total ammo count" dataDxfId="0">
+    <tableColumn id="10" xr3:uid="{3136763A-E7B4-4737-8D7B-5551B327F9C1}" name="Total ammo count" dataDxfId="3">
       <calculatedColumnFormula>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{2E765636-6761-4DD2-AC4B-A67DB815DB20}" name="DPS" dataDxfId="4">
+    <tableColumn id="5" xr3:uid="{2E765636-6761-4DD2-AC4B-A67DB815DB20}" name="DPS" dataDxfId="2">
       <calculatedColumnFormula>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{EB559151-FD07-4F49-B080-7CD123C7CBB5}" name="Damage per mag" dataDxfId="3">
+    <tableColumn id="7" xr3:uid="{EB559151-FD07-4F49-B080-7CD123C7CBB5}" name="Damage per mag" dataDxfId="1">
       <calculatedColumnFormula>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2D973EAE-7FBD-4D23-A593-979D1D4AD654}" name="Damage per rearm" dataDxfId="2">
+    <tableColumn id="9" xr3:uid="{2D973EAE-7FBD-4D23-A593-979D1D4AD654}" name="Damage per rearm" dataDxfId="0">
       <calculatedColumnFormula>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -524,11 +523,11 @@
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
         <v>50</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2">
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
         <v>500</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2">
         <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
         <v>2500</v>
       </c>
@@ -564,11 +563,11 @@
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
         <v>583.33333333333337</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3">
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
         <v>875</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3">
         <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
         <v>5250</v>
       </c>
@@ -604,11 +603,11 @@
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
         <v>400</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4">
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
         <v>600</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4">
         <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
         <v>2400</v>
       </c>
@@ -644,11 +643,11 @@
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
         <v>125</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5">
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
         <v>375</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5">
         <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
         <v>2625</v>
       </c>

</xml_diff>

<commit_message>
Slightly rebalanced weapons and enemies
</commit_message>
<xml_diff>
--- a/Assets/Spreadsheets/GunBalancing.xlsx
+++ b/Assets/Spreadsheets/GunBalancing.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zilant\Unity Projects SSD\Jam Game\Assets\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D6A73A9-453B-4A2D-A313-B3EEBA8C5702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9010977-45C8-48D3-8B93-CA76D475909B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="375" yWindow="2055" windowWidth="28800" windowHeight="18450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2775" yWindow="3000" windowWidth="24210" windowHeight="9285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Name</t>
   </si>
@@ -81,6 +81,27 @@
   </si>
   <si>
     <t>Spare ammo count</t>
+  </si>
+  <si>
+    <t>AR</t>
+  </si>
+  <si>
+    <t>Bolter</t>
+  </si>
+  <si>
+    <t>GL</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>Revolver</t>
+  </si>
+  <si>
+    <t>Super Shotgun</t>
+  </si>
+  <si>
+    <t>Auto Shotgun</t>
   </si>
 </sst>
 </file>
@@ -116,8 +137,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -152,8 +174,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A6E1795C-B8BE-4D83-98EB-3638F860B024}" name="Table1" displayName="Table1" ref="A1:K5" totalsRowShown="0">
-  <autoFilter ref="A1:K5" xr:uid="{A6E1795C-B8BE-4D83-98EB-3638F860B024}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A6E1795C-B8BE-4D83-98EB-3638F860B024}" name="Table1" displayName="Table1" ref="A1:K12" totalsRowShown="0">
+  <autoFilter ref="A1:K12" xr:uid="{A6E1795C-B8BE-4D83-98EB-3638F860B024}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K12">
+    <sortCondition descending="1" ref="K1:K12"/>
+  </sortState>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{1A0B763C-6775-455F-A197-9AB6F519E7CD}" name="Name"/>
     <tableColumn id="2" xr3:uid="{A05A5E0A-535D-4FF7-A7DF-E8BA034DF865}" name="Damage/Bullet"/>
@@ -444,9 +469,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" customWidth="1"/>
     <col min="4" max="4" width="14.140625" customWidth="1"/>
@@ -455,6 +481,8 @@
     <col min="7" max="7" width="20.42578125" customWidth="1"/>
     <col min="8" max="8" width="19.42578125" customWidth="1"/>
     <col min="9" max="9" width="21" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -494,162 +522,442 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B2">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F2">
         <v>5</v>
       </c>
-      <c r="G2">
-        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
-        <v>25</v>
-      </c>
-      <c r="H2">
-        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+      <c r="G2" s="1">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
         <v>30</v>
       </c>
-      <c r="I2">
-        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
-        <v>50</v>
-      </c>
-      <c r="J2">
-        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
-        <v>500</v>
-      </c>
-      <c r="K2">
-        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
-        <v>2500</v>
+      <c r="H2" s="1">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>36</v>
+      </c>
+      <c r="I2" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>600</v>
+      </c>
+      <c r="J2" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>1800</v>
+      </c>
+      <c r="K2" s="1">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>9000</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B3">
         <v>25</v>
       </c>
       <c r="C3">
-        <v>0.3</v>
+        <v>7.5999999999999998E-2</v>
       </c>
       <c r="D3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="F3">
-        <v>6</v>
-      </c>
-      <c r="G3">
-        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
-        <v>30</v>
-      </c>
-      <c r="H3">
-        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
-        <v>35</v>
-      </c>
-      <c r="I3">
-        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
-        <v>583.33333333333337</v>
-      </c>
-      <c r="J3">
-        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
-        <v>875</v>
-      </c>
-      <c r="K3">
-        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
-        <v>5250</v>
+        <v>3</v>
+      </c>
+      <c r="G3" s="1">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>300</v>
+      </c>
+      <c r="H3" s="1">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>400</v>
+      </c>
+      <c r="I3" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>328.94736842105266</v>
+      </c>
+      <c r="J3" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>2500</v>
+      </c>
+      <c r="K3" s="1">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>7500</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B4">
+        <v>15</v>
+      </c>
+      <c r="C4">
+        <v>0.3</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
         <v>20</v>
       </c>
-      <c r="C4">
-        <v>0.05</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>30</v>
-      </c>
       <c r="F4">
-        <v>4</v>
-      </c>
-      <c r="G4">
-        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>5</v>
+      </c>
+      <c r="G4" s="1">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>100</v>
+      </c>
+      <c r="H4" s="1">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
         <v>120</v>
       </c>
-      <c r="H4">
-        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
-        <v>150</v>
-      </c>
-      <c r="I4">
-        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
-        <v>400</v>
-      </c>
-      <c r="J4">
-        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
-        <v>600</v>
-      </c>
-      <c r="K4">
-        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
-        <v>2400</v>
+      <c r="I4" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>250</v>
+      </c>
+      <c r="J4" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>1500</v>
+      </c>
+      <c r="K4" s="1">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>7500</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="B5">
         <v>25</v>
       </c>
       <c r="C5">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="D5">
+        <v>14</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>10</v>
+      </c>
+      <c r="G5" s="1">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>20</v>
+      </c>
+      <c r="H5" s="1">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>22</v>
+      </c>
+      <c r="I5" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>388.88888888888886</v>
+      </c>
+      <c r="J5" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>700</v>
+      </c>
+      <c r="K5" s="1">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>15</v>
+      </c>
+      <c r="C6">
+        <v>0.3</v>
+      </c>
+      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6">
+        <v>6</v>
+      </c>
+      <c r="G6">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>30</v>
+      </c>
+      <c r="H6">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>35</v>
+      </c>
+      <c r="I6">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>350</v>
+      </c>
+      <c r="J6">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>525</v>
+      </c>
+      <c r="K6">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>3150</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>34</v>
+      </c>
+      <c r="C7">
+        <v>0.1</v>
+      </c>
+      <c r="D7">
         <v>1</v>
       </c>
-      <c r="E5">
+      <c r="E7">
+        <v>30</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7" s="1">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>150</v>
+      </c>
+      <c r="H7" s="1">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>180</v>
+      </c>
+      <c r="I7" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>340</v>
+      </c>
+      <c r="J7" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>1020</v>
+      </c>
+      <c r="K7" s="1">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>5100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8">
+        <v>200</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>5</v>
+      </c>
+      <c r="F8">
+        <v>5</v>
+      </c>
+      <c r="G8">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>25</v>
+      </c>
+      <c r="H8">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>30</v>
+      </c>
+      <c r="I8">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>100</v>
+      </c>
+      <c r="J8">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>1000</v>
+      </c>
+      <c r="K8">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>25</v>
+      </c>
+      <c r="C9">
+        <v>0.05</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
         <v>15</v>
       </c>
-      <c r="F5">
+      <c r="F9">
+        <v>10</v>
+      </c>
+      <c r="G9">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>150</v>
+      </c>
+      <c r="H9">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>165</v>
+      </c>
+      <c r="I9">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>500</v>
+      </c>
+      <c r="J9">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>375</v>
+      </c>
+      <c r="K9">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>3750</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>7</v>
       </c>
-      <c r="G5">
-        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
-        <v>105</v>
-      </c>
-      <c r="H5">
-        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
-        <v>120</v>
-      </c>
-      <c r="I5">
-        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
-        <v>125</v>
-      </c>
-      <c r="J5">
-        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
-        <v>375</v>
-      </c>
-      <c r="K5">
-        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
-        <v>2625</v>
+      <c r="B10">
+        <v>25</v>
+      </c>
+      <c r="C10">
+        <v>0.05</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>30</v>
+      </c>
+      <c r="F10">
+        <v>5</v>
+      </c>
+      <c r="G10">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>150</v>
+      </c>
+      <c r="H10">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>180</v>
+      </c>
+      <c r="I10">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>500</v>
+      </c>
+      <c r="J10">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>750</v>
+      </c>
+      <c r="K10">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>3750</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
+        <v>75</v>
+      </c>
+      <c r="C11">
+        <v>0.5</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>10</v>
+      </c>
+      <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11" s="1">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>40</v>
+      </c>
+      <c r="H11" s="1">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>50</v>
+      </c>
+      <c r="I11" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>150</v>
+      </c>
+      <c r="J11" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>750</v>
+      </c>
+      <c r="K11" s="1">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
+        <v>200</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+      <c r="G12" s="1">
+        <f>Table1[[#This Row],[Mag size]]*Table1[[#This Row],[Mag count]]</f>
+        <v>10</v>
+      </c>
+      <c r="H12" s="1">
+        <f>Table1[[#This Row],[Mag size]]+Table1[[#This Row],[Spare ammo count]]</f>
+        <v>11</v>
+      </c>
+      <c r="I12" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
+        <v>100</v>
+      </c>
+      <c r="J12" s="1">
+        <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
+        <v>200</v>
+      </c>
+      <c r="K12" s="1">
+        <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed UI placement and made a level template
</commit_message>
<xml_diff>
--- a/Assets/Spreadsheets/GunBalancing.xlsx
+++ b/Assets/Spreadsheets/GunBalancing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zilant\Unity Projects SSD\Jam Game\Assets\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9010977-45C8-48D3-8B93-CA76D475909B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5B5B42-F7E1-4AA9-BD9F-A66DDD822C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2775" yWindow="3000" windowWidth="24210" windowHeight="9285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -685,7 +685,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C6">
         <v>0.3</v>
@@ -709,15 +709,15 @@
       </c>
       <c r="I6">
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]/Table1[[#This Row],[Fire rate]]</f>
-        <v>350</v>
+        <v>466.66666666666669</v>
       </c>
       <c r="J6">
         <f>Table1[[#This Row],[Damage/Bullet]]*Table1[[#This Row],[Bullets/Shot]]*Table1[[#This Row],[Mag size]]</f>
-        <v>525</v>
+        <v>700</v>
       </c>
       <c r="K6">
         <f>Table1[[#This Row],[Damage per mag]]*Table1[[#This Row],[Mag count]]</f>
-        <v>3150</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>